<commit_message>
chore: publish homecareobservation IG 1.2.2
</commit_message>
<xml_diff>
--- a/ig/homecareobservation/StructureDefinition-medcom-homecare-observation.xlsx
+++ b/ig/homecareobservation/StructureDefinition-medcom-homecare-observation.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.1</t>
+    <t>1.2.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-19T07:53:40+00:00</t>
+    <t>2026-06-03T08:12:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -3412,7 +3412,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" hidden="true">
+    <row r="7">
       <c r="A7" t="s" s="2">
         <v>120</v>
       </c>
@@ -4254,7 +4254,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" hidden="true">
+    <row r="14">
       <c r="A14" t="s" s="2">
         <v>176</v>
       </c>
@@ -4496,7 +4496,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" hidden="true">
+    <row r="16">
       <c r="A16" t="s" s="2">
         <v>198</v>
       </c>
@@ -5214,7 +5214,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" hidden="true">
+    <row r="22">
       <c r="A22" t="s" s="2">
         <v>237</v>
       </c>
@@ -5456,7 +5456,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" hidden="true">
+    <row r="24">
       <c r="A24" t="s" s="2">
         <v>252</v>
       </c>
@@ -5576,7 +5576,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" hidden="true">
+    <row r="25">
       <c r="A25" t="s" s="2">
         <v>259</v>
       </c>
@@ -6180,7 +6180,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" hidden="true">
+    <row r="30">
       <c r="A30" t="s" s="2">
         <v>280</v>
       </c>
@@ -6422,7 +6422,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" hidden="true">
+    <row r="32">
       <c r="A32" t="s" s="2">
         <v>283</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" hidden="true">
+    <row r="33">
       <c r="A33" t="s" s="2">
         <v>284</v>
       </c>
@@ -7146,7 +7146,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="38" hidden="true">
+    <row r="38">
       <c r="A38" t="s" s="2">
         <v>291</v>
       </c>
@@ -7388,7 +7388,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="40" hidden="true">
+    <row r="40">
       <c r="A40" t="s" s="2">
         <v>294</v>
       </c>
@@ -7508,7 +7508,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="41" hidden="true">
+    <row r="41">
       <c r="A41" t="s" s="2">
         <v>295</v>
       </c>
@@ -8112,7 +8112,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" hidden="true">
+    <row r="46">
       <c r="A46" t="s" s="2">
         <v>302</v>
       </c>
@@ -8354,7 +8354,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="48" hidden="true">
+    <row r="48">
       <c r="A48" t="s" s="2">
         <v>305</v>
       </c>
@@ -8472,7 +8472,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="49" hidden="true">
+    <row r="49">
       <c r="A49" t="s" s="2">
         <v>307</v>
       </c>
@@ -9076,7 +9076,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="54" hidden="true">
+    <row r="54">
       <c r="A54" t="s" s="2">
         <v>314</v>
       </c>
@@ -9318,7 +9318,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="56" hidden="true">
+    <row r="56">
       <c r="A56" t="s" s="2">
         <v>317</v>
       </c>
@@ -9438,7 +9438,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="57" hidden="true">
+    <row r="57">
       <c r="A57" t="s" s="2">
         <v>318</v>
       </c>
@@ -10042,7 +10042,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="62" hidden="true">
+    <row r="62">
       <c r="A62" t="s" s="2">
         <v>324</v>
       </c>
@@ -10284,7 +10284,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="64" hidden="true">
+    <row r="64">
       <c r="A64" t="s" s="2">
         <v>327</v>
       </c>
@@ -10402,7 +10402,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="65" hidden="true">
+    <row r="65">
       <c r="A65" t="s" s="2">
         <v>329</v>
       </c>
@@ -11006,7 +11006,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="70" hidden="true">
+    <row r="70">
       <c r="A70" t="s" s="2">
         <v>336</v>
       </c>
@@ -11248,7 +11248,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="72" hidden="true">
+    <row r="72">
       <c r="A72" t="s" s="2">
         <v>339</v>
       </c>
@@ -11368,7 +11368,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="73" hidden="true">
+    <row r="73">
       <c r="A73" t="s" s="2">
         <v>340</v>
       </c>
@@ -11732,7 +11732,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" hidden="true">
+    <row r="76">
       <c r="A76" t="s" s="2">
         <v>350</v>
       </c>
@@ -12216,7 +12216,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="80" hidden="true">
+    <row r="80">
       <c r="A80" t="s" s="2">
         <v>389</v>
       </c>
@@ -12700,7 +12700,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="84" hidden="true">
+    <row r="84">
       <c r="A84" t="s" s="2">
         <v>422</v>
       </c>
@@ -13062,7 +13062,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="87" hidden="true">
+    <row r="87">
       <c r="A87" t="s" s="2">
         <v>429</v>
       </c>
@@ -13668,7 +13668,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="92" hidden="true">
+    <row r="92">
       <c r="A92" t="s" s="2">
         <v>476</v>
       </c>
@@ -13914,7 +13914,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="94" hidden="true">
+    <row r="94">
       <c r="A94" t="s" s="2">
         <v>488</v>
       </c>
@@ -15358,7 +15358,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="106" hidden="true">
+    <row r="106">
       <c r="A106" t="s" s="2">
         <v>511</v>
       </c>
@@ -27182,12 +27182,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AP203">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
chore: publish homecareobservation IG 1.2.2 (#81)
Co-authored-by: tmsMedcom <tmsMedcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/homecareobservation/StructureDefinition-medcom-homecare-observation.xlsx
+++ b/ig/homecareobservation/StructureDefinition-medcom-homecare-observation.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.1</t>
+    <t>1.2.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-19T07:53:40+00:00</t>
+    <t>2026-06-03T08:12:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -3412,7 +3412,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" hidden="true">
+    <row r="7">
       <c r="A7" t="s" s="2">
         <v>120</v>
       </c>
@@ -4254,7 +4254,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" hidden="true">
+    <row r="14">
       <c r="A14" t="s" s="2">
         <v>176</v>
       </c>
@@ -4496,7 +4496,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" hidden="true">
+    <row r="16">
       <c r="A16" t="s" s="2">
         <v>198</v>
       </c>
@@ -5214,7 +5214,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" hidden="true">
+    <row r="22">
       <c r="A22" t="s" s="2">
         <v>237</v>
       </c>
@@ -5456,7 +5456,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" hidden="true">
+    <row r="24">
       <c r="A24" t="s" s="2">
         <v>252</v>
       </c>
@@ -5576,7 +5576,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" hidden="true">
+    <row r="25">
       <c r="A25" t="s" s="2">
         <v>259</v>
       </c>
@@ -6180,7 +6180,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" hidden="true">
+    <row r="30">
       <c r="A30" t="s" s="2">
         <v>280</v>
       </c>
@@ -6422,7 +6422,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" hidden="true">
+    <row r="32">
       <c r="A32" t="s" s="2">
         <v>283</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" hidden="true">
+    <row r="33">
       <c r="A33" t="s" s="2">
         <v>284</v>
       </c>
@@ -7146,7 +7146,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="38" hidden="true">
+    <row r="38">
       <c r="A38" t="s" s="2">
         <v>291</v>
       </c>
@@ -7388,7 +7388,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="40" hidden="true">
+    <row r="40">
       <c r="A40" t="s" s="2">
         <v>294</v>
       </c>
@@ -7508,7 +7508,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="41" hidden="true">
+    <row r="41">
       <c r="A41" t="s" s="2">
         <v>295</v>
       </c>
@@ -8112,7 +8112,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" hidden="true">
+    <row r="46">
       <c r="A46" t="s" s="2">
         <v>302</v>
       </c>
@@ -8354,7 +8354,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="48" hidden="true">
+    <row r="48">
       <c r="A48" t="s" s="2">
         <v>305</v>
       </c>
@@ -8472,7 +8472,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="49" hidden="true">
+    <row r="49">
       <c r="A49" t="s" s="2">
         <v>307</v>
       </c>
@@ -9076,7 +9076,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="54" hidden="true">
+    <row r="54">
       <c r="A54" t="s" s="2">
         <v>314</v>
       </c>
@@ -9318,7 +9318,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="56" hidden="true">
+    <row r="56">
       <c r="A56" t="s" s="2">
         <v>317</v>
       </c>
@@ -9438,7 +9438,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="57" hidden="true">
+    <row r="57">
       <c r="A57" t="s" s="2">
         <v>318</v>
       </c>
@@ -10042,7 +10042,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="62" hidden="true">
+    <row r="62">
       <c r="A62" t="s" s="2">
         <v>324</v>
       </c>
@@ -10284,7 +10284,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="64" hidden="true">
+    <row r="64">
       <c r="A64" t="s" s="2">
         <v>327</v>
       </c>
@@ -10402,7 +10402,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="65" hidden="true">
+    <row r="65">
       <c r="A65" t="s" s="2">
         <v>329</v>
       </c>
@@ -11006,7 +11006,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="70" hidden="true">
+    <row r="70">
       <c r="A70" t="s" s="2">
         <v>336</v>
       </c>
@@ -11248,7 +11248,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="72" hidden="true">
+    <row r="72">
       <c r="A72" t="s" s="2">
         <v>339</v>
       </c>
@@ -11368,7 +11368,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="73" hidden="true">
+    <row r="73">
       <c r="A73" t="s" s="2">
         <v>340</v>
       </c>
@@ -11732,7 +11732,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" hidden="true">
+    <row r="76">
       <c r="A76" t="s" s="2">
         <v>350</v>
       </c>
@@ -12216,7 +12216,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="80" hidden="true">
+    <row r="80">
       <c r="A80" t="s" s="2">
         <v>389</v>
       </c>
@@ -12700,7 +12700,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="84" hidden="true">
+    <row r="84">
       <c r="A84" t="s" s="2">
         <v>422</v>
       </c>
@@ -13062,7 +13062,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="87" hidden="true">
+    <row r="87">
       <c r="A87" t="s" s="2">
         <v>429</v>
       </c>
@@ -13668,7 +13668,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="92" hidden="true">
+    <row r="92">
       <c r="A92" t="s" s="2">
         <v>476</v>
       </c>
@@ -13914,7 +13914,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="94" hidden="true">
+    <row r="94">
       <c r="A94" t="s" s="2">
         <v>488</v>
       </c>
@@ -15358,7 +15358,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="106" hidden="true">
+    <row r="106">
       <c r="A106" t="s" s="2">
         <v>511</v>
       </c>
@@ -27182,12 +27182,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AP203">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>